<commit_message>
-se genero la automatización de las recoleccion de las metricas de concuncurrencia desde un archivo excel al excel automatico
</commit_message>
<xml_diff>
--- a/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Resultado_uso_de_Memoria.xlsx
+++ b/metricas_realizadas/Prog-Concurrente/Analisis de metricas/Resultado_uso_de_Memoria.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyecto_code_ia\metricas_realizadas\Prog-Concurrente\Analisis de metricas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBA44BE5-8E37-445C-A50A-3DE9A4D0AEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E85FD0-37C1-4A71-A2F6-2BA6A903C8D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="51">
   <si>
     <t>Grupo</t>
   </si>
@@ -186,6 +186,12 @@
   </si>
   <si>
     <t>Las configuraciones evaluadas por el grupo M4 presentaron los menores consumos de memoria, mientras que las correspondientes al grupo M6 registraron los mayores valores.</t>
+  </si>
+  <si>
+    <t>Claude Sonnet 4.6 +opus</t>
+  </si>
+  <si>
+    <t>Haiku 4.5+opus+sonnet</t>
   </si>
 </sst>
 </file>
@@ -194,7 +200,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -284,7 +290,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -293,16 +299,11 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -355,17 +356,17 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1158,7 +1159,7 @@
                 <c:formatCode>_-* #,##0_-;\-* #,##0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>68</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1515,7 +1516,7 @@
                 <c:formatCode>_-* #,##0_-;\-* #,##0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>200</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1992,7 +1993,7 @@
                 <c:formatCode>_-* #,##0_-;\-* #,##0_-;_-* "-"??_-;_-@_-</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>396</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3048,7 +3049,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" customWidth="1"/>
@@ -3095,320 +3096,254 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="13">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="7">
         <v>52</v>
       </c>
-      <c r="I2" s="5"/>
+      <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="13" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="H3" s="7">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="28"/>
+      <c r="C4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" s="13">
+        <v>0.42</v>
+      </c>
+      <c r="H4" s="7">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="27"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0.42</v>
+      </c>
+      <c r="H5" s="7">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F6" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="16">
-        <v>0.5</v>
-      </c>
-      <c r="H3" s="10">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="G6" s="20">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="H6" s="11">
+        <v>20</v>
+      </c>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F7" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="16">
-        <v>0.5</v>
-      </c>
-      <c r="H4" s="10">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="29"/>
-      <c r="C5" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="G5" s="16">
-        <v>0.42</v>
-      </c>
-      <c r="H5" s="10">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="16">
-        <v>0.42</v>
-      </c>
-      <c r="H6" s="10">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="23">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="H7" s="14">
-        <v>20</v>
-      </c>
-      <c r="I7" s="9"/>
+      <c r="G7" s="20">
+        <v>2E-3</v>
+      </c>
+      <c r="H7" s="7">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="23">
-        <v>2E-3</v>
-      </c>
-      <c r="H8" s="10">
-        <v>15</v>
+      <c r="G8" s="21">
+        <v>0.1061</v>
+      </c>
+      <c r="H8" s="7">
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="9" t="s">
+      <c r="D9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="24">
-        <v>0.1061</v>
-      </c>
-      <c r="H9" s="10">
+      <c r="G9" s="21">
+        <v>0.12429999999999999</v>
+      </c>
+      <c r="H9" s="7">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="2"/>
-      <c r="B10" s="5" t="s">
-        <v>32</v>
+      <c r="A10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="G10" s="24">
-        <v>0.12429999999999999</v>
-      </c>
-      <c r="H10" s="10">
-        <v>20</v>
-      </c>
+      <c r="F10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="20">
+        <v>2.0333000000000001</v>
+      </c>
+      <c r="H10" s="22">
+        <v>200</v>
+      </c>
+      <c r="I10" s="12"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="8" t="s">
         <v>10</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="6" t="s">
-        <v>36</v>
+      <c r="F11" s="10" t="s">
+        <v>37</v>
       </c>
       <c r="G11" s="23">
-        <v>2.0333000000000001</v>
-      </c>
-      <c r="H11" s="25">
-        <v>200</v>
-      </c>
-      <c r="I11" s="15"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="3"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="G12" s="23">
-        <v>2.0333000000000001</v>
-      </c>
-      <c r="H12" s="25">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="26">
         <v>3.04</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H11" s="7">
         <v>396</v>
       </c>
-      <c r="I13" s="15"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="4"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="G14" s="26">
-        <v>3.04</v>
-      </c>
-      <c r="H14" s="10">
-        <v>396</v>
-      </c>
+      <c r="I11" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3426,259 +3361,259 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="17" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="30">
+      <c r="D2" s="25">
+        <f>'CPU y memoria'!H7</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="25">
+        <f>'CPU y memoria'!H6</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="25">
         <f>'CPU y memoria'!H8</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B5" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="30">
-        <f>'CPU y memoria'!H7</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D4" s="30">
+      <c r="C5" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="25">
         <f>'CPU y memoria'!H9</f>
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="30">
-        <f>'CPU y memoria'!H10</f>
-        <v>20</v>
-      </c>
-    </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="19" t="s">
+      <c r="C6" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="26">
         <f>'CPU y memoria'!H2</f>
         <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="31">
-        <f>'CPU y memoria'!H4</f>
-        <v>68</v>
+      <c r="D7" s="26" t="e">
+        <f>'CPU y memoria'!#REF!</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="26">
         <f>'CPU y memoria'!H3</f>
         <v>68</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="30">
+      <c r="D9" s="25">
+        <f>'CPU y memoria'!H10</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="25" t="e">
+        <f>'CPU y memoria'!#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="26">
+        <f>'CPU y memoria'!H4</f>
+        <v>238</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="26">
+        <f>'CPU y memoria'!H4</f>
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="25">
         <f>'CPU y memoria'!H11</f>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="19" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="25" t="e">
+        <f>'CPU y memoria'!#REF!</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" s="30">
-        <f>'CPU y memoria'!H12</f>
-        <v>200</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+      <c r="B19" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="31">
-        <f>'CPU y memoria'!H5</f>
-        <v>238</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D12" s="31">
-        <f>'CPU y memoria'!H5</f>
-        <v>238</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="30">
-        <f>'CPU y memoria'!H13</f>
-        <v>396</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="19" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="30">
-        <f>'CPU y memoria'!H14</f>
-        <v>396</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17" s="17" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="21" t="s">
-        <v>3</v>
-      </c>
-      <c r="B18" s="17" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>42</v>
       </c>
     </row>
@@ -3699,84 +3634,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J1" s="27" t="s">
+      <c r="J1" s="24" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="15" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J3" s="21" t="s">
+      <c r="J3" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="K3" s="14" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J4" s="21" t="s">
+      <c r="J4" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="17" t="s">
+      <c r="K4" s="14" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="5" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J5" s="21" t="s">
+      <c r="J5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="14" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J6" s="21" t="s">
+      <c r="J6" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="14" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="7" spans="10:11" x14ac:dyDescent="0.35">
-      <c r="J7" s="21" t="s">
+      <c r="J7" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="14" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B24" s="22"/>
+      <c r="B24" s="19"/>
     </row>
     <row r="25" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="19" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B26" s="12"/>
+      <c r="B26" s="9"/>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="19" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="19" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B29" s="12"/>
+      <c r="B29" s="9"/>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="19" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>